<commit_message>
fix(R2): corregir precisión de Base Gravable al evitar conversión MXN->USD->MXN
</commit_message>
<xml_diff>
--- a/catalogos/FechaDOF.xlsx
+++ b/catalogos/FechaDOF.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B172"/>
+  <dimension ref="A1:B173"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1760,6 +1760,14 @@
         <v>17.7228</v>
       </c>
     </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="2">
+        <v>46086</v>
+      </c>
+      <c r="B173">
+        <v>17.5445</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add 4b_Facturas Exportacion tab filtering by Tipo Operacion
</commit_message>
<xml_diff>
--- a/catalogos/FechaDOF.xlsx
+++ b/catalogos/FechaDOF.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B173"/>
+  <dimension ref="A1:B175"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1768,6 +1768,22 @@
         <v>17.5445</v>
       </c>
     </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="2">
+        <v>46087</v>
+      </c>
+      <c r="B174">
+        <v>17.677</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="2">
+        <v>46090</v>
+      </c>
+      <c r="B175">
+        <v>17.7962</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: mejoras en persistencia, parser de ZIPs y etiquetas
- Se condiciona la inserción a BD según la variable ENVIRONMENT (solo if produccion)
- Mejoras en asc_parser para soportar extracción de ZIPs anidados y múltiples Excel
- Se actualiza la etiqueta 'Delta' por 'Diferencia Total vs DataStage' en Reporte 2
</commit_message>
<xml_diff>
--- a/catalogos/FechaDOF.xlsx
+++ b/catalogos/FechaDOF.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B175"/>
+  <dimension ref="A1:B178"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1784,6 +1784,30 @@
         <v>17.7962</v>
       </c>
     </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="2">
+        <v>46091</v>
+      </c>
+      <c r="B176">
+        <v>17.7687</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="2">
+        <v>46092</v>
+      </c>
+      <c r="B177">
+        <v>17.5037</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="2">
+        <v>46093</v>
+      </c>
+      <c r="B178">
+        <v>17.6543</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>